<commit_message>
Remove substrate_1_id in favour of substrate_id
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_results/lanupro_vocabulary_incubations.xlsx
+++ b/data/raw_results/lanupro_vocabulary_incubations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my_github_projects\lanupro_vocabulary_2025\data\raw_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924E4365-7A99-4895-BD7E-D9416ABC8C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7F43F5-6E6B-4196-8C12-BEC699D74FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7197A02B-EEB4-4DD3-A670-5499E50D1EFE}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </externalReferences>
   <definedNames>
     <definedName name="Analyst">#REF!:INDEX(#REF!,COUNTA(#REF!))</definedName>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">vocabulary!$A:$CO</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">vocabulary!$A:$CN</definedName>
     <definedName name="factor_dropdown">IF(_xlfn.XLOOKUP([1]scientific_sheet!A$1,[1]!lanupro_vocabulary_combined[#Headers],INDEX([1]!lanupro_vocabulary_combined[#Data],MATCH("type",[1]!lanupro_vocabulary_combined[lanupro_ontology],0),0))="factor",INDIRECT("lanupro_vocabulary_combined["&amp;[1]scientific_sheet!A$1&amp;"]"),"")</definedName>
     <definedName name="GC">#REF!:INDEX(#REF!,COUNTA(#REF!))</definedName>
     <definedName name="GC_method">#REF!:INDEX(#REF!,COUNTA(#REF!))</definedName>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10166" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10060" uniqueCount="344">
   <si>
     <t>lanupro_ontology</t>
   </si>
@@ -695,13 +695,7 @@
     <t>type of inocula used</t>
   </si>
   <si>
-    <t>id of the substrate</t>
-  </si>
-  <si>
     <t>amount of substrate added (mg)</t>
-  </si>
-  <si>
-    <t>substrate_1_id</t>
   </si>
   <si>
     <t>substrate_1_type</t>
@@ -1433,7 +1427,7 @@
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{CE8575D7-D81A-4D4D-BBF6-CFACC4DABE43}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="107" unboundColumnsRight="3">
-    <queryTableFields count="96">
+    <queryTableFields count="95">
       <queryTableField id="1" name="lanupro_ontology" tableColumnId="1"/>
       <queryTableField id="2" name="substrate_ms_id" tableColumnId="2"/>
       <queryTableField id="3" name="substrate_ms_mg" tableColumnId="3"/>
@@ -1459,7 +1453,6 @@
       <queryTableField id="101" dataBound="0" tableColumnId="91"/>
       <queryTableField id="102" dataBound="0" tableColumnId="92"/>
       <queryTableField id="81" dataBound="0" tableColumnId="79"/>
-      <queryTableField id="88" dataBound="0" tableColumnId="70"/>
       <queryTableField id="82" dataBound="0" tableColumnId="80"/>
       <queryTableField id="89" dataBound="0" tableColumnId="73"/>
       <queryTableField id="15" name="trt" tableColumnId="15"/>
@@ -1536,9 +1529,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0B81B339-58BA-4A96-9675-10230FA0D708}" name="lanupro_vocabulary_incubations" displayName="lanupro_vocabulary_incubations" ref="A1:CR1048576" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:CR1048576" xr:uid="{681020AF-0257-46A7-AFB6-6083C8C339F0}"/>
-  <tableColumns count="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0B81B339-58BA-4A96-9675-10230FA0D708}" name="lanupro_vocabulary_incubations" displayName="lanupro_vocabulary_incubations" ref="A1:CQ1048576" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:CQ1048576" xr:uid="{681020AF-0257-46A7-AFB6-6083C8C339F0}"/>
+  <tableColumns count="95">
     <tableColumn id="1" xr3:uid="{E0057884-D0FA-4191-B40E-09169C0C7C3C}" uniqueName="1" name="lanupro_ontology" queryTableFieldId="1" dataDxfId="74"/>
     <tableColumn id="2" xr3:uid="{ED720914-91FC-4824-BA54-EA1390DD6AAF}" uniqueName="2" name="substrate_ms_id" queryTableFieldId="2" dataDxfId="73"/>
     <tableColumn id="3" xr3:uid="{C98FD6B0-6BB8-4D25-A1B9-C08CD2891DFE}" uniqueName="3" name="substrate_ms_mg" queryTableFieldId="3" dataDxfId="72"/>
@@ -1564,7 +1557,6 @@
     <tableColumn id="91" xr3:uid="{4C65E12D-86B9-473B-A866-FE3129457F9C}" uniqueName="91" name="cow_ilvo_id" queryTableFieldId="101"/>
     <tableColumn id="92" xr3:uid="{B28188A6-01B4-4D1F-A64D-7AE40B7F5845}" uniqueName="92" name="diet_cows" queryTableFieldId="102"/>
     <tableColumn id="79" xr3:uid="{5DDB981D-3A78-45F3-8EC2-94928028E554}" uniqueName="79" name="inocula_type" queryTableFieldId="81"/>
-    <tableColumn id="70" xr3:uid="{650A2099-A092-4C7B-9B62-F9243FBBA9D1}" uniqueName="70" name="substrate_1_id" queryTableFieldId="88"/>
     <tableColumn id="80" xr3:uid="{A01C1450-87EF-47A3-9093-B7C7EACE4000}" uniqueName="80" name="substrate_1_type" queryTableFieldId="82"/>
     <tableColumn id="73" xr3:uid="{F985F988-5F8F-4A6F-8482-53D9E7052230}" uniqueName="73" name="substrate_1_mg" queryTableFieldId="89"/>
     <tableColumn id="15" xr3:uid="{6C1AE535-1B92-4BEE-A9B7-C36F9C205E82}" uniqueName="15" name="trt_label_1" queryTableFieldId="15" dataDxfId="63"/>
@@ -1927,7 +1919,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7482448-506A-411A-B0FB-59A8EF966460}">
-  <dimension ref="A1:CR106"/>
+  <dimension ref="A1:CQ106"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
@@ -1940,72 +1932,72 @@
     <col min="8" max="19" width="62.33203125" customWidth="1"/>
     <col min="20" max="20" width="74.44140625" bestFit="1" customWidth="1"/>
     <col min="21" max="24" width="46.21875" bestFit="1" customWidth="1"/>
-    <col min="25" max="28" width="46.21875" customWidth="1"/>
-    <col min="29" max="29" width="33.33203125" customWidth="1"/>
-    <col min="30" max="31" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="72.33203125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="70.21875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="34.77734375" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="35.109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="35.109375" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="35.109375" bestFit="1" customWidth="1"/>
-    <col min="46" max="47" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="35.109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="51" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="30" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="65" max="66" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="21.77734375" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="23.5546875" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="21" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="20" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="16" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="28.44140625" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="28.5546875" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="30.109375" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="30.88671875" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="80.5546875" customWidth="1"/>
-    <col min="95" max="95" width="27" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="27" width="46.21875" customWidth="1"/>
+    <col min="28" max="28" width="33.33203125" customWidth="1"/>
+    <col min="29" max="30" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="72.33203125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="70.21875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="34.77734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="50" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="30" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="35.21875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="64" max="65" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="21" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="20" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="16" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="28.44140625" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="30.88671875" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="80.5546875" customWidth="1"/>
+    <col min="94" max="94" width="27" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="22.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:96">
+    <row r="1" spans="1:95">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2034,34 +2026,34 @@
         <v>206</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>225</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>227</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>203</v>
@@ -2070,232 +2062,229 @@
         <v>204</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>228</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>230</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>202</v>
       </c>
       <c r="Z1" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="AD1" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="AE1" s="1" t="s">
-        <v>216</v>
+        <v>7</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>8</v>
+        <v>229</v>
       </c>
       <c r="AH1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="AN1" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="AI1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AP1" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="AN1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AR1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="AP1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="AT1" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="AR1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AV1" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="AT1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AX1" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="AV1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="BB1" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="AX1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AY1" s="1" t="s">
+      <c r="BC1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="BE1" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="BB1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BF1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="BD1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="BF1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="BG1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="BL1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="BM1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="BN1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="BO1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="BP1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="BR1" s="1" t="s">
+      <c r="BS1" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="BS1" s="1" t="s">
+      <c r="BT1" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="BT1" s="1" t="s">
+      <c r="BU1" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="BU1" s="1" t="s">
+      <c r="BV1" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="BV1" s="1" t="s">
+      <c r="BW1" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="BW1" s="1" t="s">
+      <c r="BX1" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="BX1" s="1" t="s">
+      <c r="BY1" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="BY1" s="1" t="s">
+      <c r="BZ1" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="BZ1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="CA1" s="1" t="s">
+      <c r="CB1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="CC1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="CD1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="CE1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="CH1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="CI1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="CJ1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="CK1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="CL1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="CM1" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CN1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="CO1" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="CC1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="CE1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="CF1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="CG1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="CH1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="CI1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="CJ1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="CK1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="CL1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="CM1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="CN1" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="CO1" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="CP1" s="1" t="s">
-        <v>253</v>
+        <v>64</v>
       </c>
       <c r="CQ1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="CR1" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:96">
+    <row r="2" spans="1:95">
       <c r="A2" s="1" t="s">
         <v>66</v>
       </c>
@@ -2339,7 +2328,7 @@
         <v>67</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="P2" s="1" t="s">
         <v>68</v>
@@ -2348,7 +2337,7 @@
         <v>67</v>
       </c>
       <c r="R2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>68</v>
@@ -2360,25 +2349,25 @@
         <v>69</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="W2" s="1" t="s">
         <v>67</v>
       </c>
       <c r="X2" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="Y2" s="1" t="s">
         <v>70</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="AA2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB2" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="AC2" s="1" t="s">
         <v>70</v>
@@ -2390,10 +2379,10 @@
         <v>70</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AH2" s="1" t="s">
         <v>68</v>
@@ -2402,61 +2391,61 @@
         <v>68</v>
       </c>
       <c r="AJ2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AK2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="AM2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AK2" s="1" t="s">
+      <c r="AN2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AL2" s="1" t="s">
+      <c r="AO2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AM2" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="AN2" s="1" t="s">
+      <c r="AP2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="AQ2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AO2" s="1" t="s">
+      <c r="AR2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AP2" s="1" t="s">
+      <c r="AS2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AQ2" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="AR2" s="1" t="s">
+      <c r="AT2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="AU2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AS2" s="1" t="s">
+      <c r="AV2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AT2" s="1" t="s">
+      <c r="AW2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AU2" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="AV2" s="1" t="s">
+      <c r="AX2" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="AY2" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="AW2" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AX2" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY2" s="1" t="s">
-        <v>254</v>
       </c>
       <c r="AZ2" s="1" t="s">
         <v>68</v>
       </c>
       <c r="BA2" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB2" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="BB2" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="BC2" s="1" t="s">
         <v>68</v>
@@ -2471,22 +2460,22 @@
         <v>68</v>
       </c>
       <c r="BG2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BH2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BH2" s="1" t="s">
+      <c r="BI2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BI2" s="1" t="s">
+      <c r="BJ2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="BJ2" s="1" t="s">
+      <c r="BK2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="BK2" s="1" t="s">
+      <c r="BL2" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="BL2" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="BM2" s="1" t="s">
         <v>68</v>
@@ -2573,19 +2562,16 @@
         <v>68</v>
       </c>
       <c r="CO2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="CP2" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="CP2" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="CQ2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="CR2" s="1" t="s">
-        <v>68</v>
-      </c>
     </row>
-    <row r="3" spans="1:96">
+    <row r="3" spans="1:95">
       <c r="A3" s="1" t="s">
         <v>71</v>
       </c>
@@ -2614,7 +2600,7 @@
         <v>72</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>72</v>
@@ -2626,37 +2612,37 @@
         <v>72</v>
       </c>
       <c r="N3" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>261</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>72</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="W3" s="1" t="s">
         <v>72</v>
       </c>
       <c r="X3" s="1" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>72</v>
@@ -2683,10 +2669,10 @@
         <v>72</v>
       </c>
       <c r="AG3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>72</v>
@@ -2695,19 +2681,19 @@
         <v>72</v>
       </c>
       <c r="AK3" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="AM3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AL3" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="AM3" s="1" t="s">
-        <v>266</v>
-      </c>
       <c r="AN3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="AO3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AO3" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="AP3" s="1" t="s">
         <v>72</v>
@@ -2716,10 +2702,10 @@
         <v>72</v>
       </c>
       <c r="AR3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AS3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AS3" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="AT3" s="1" t="s">
         <v>72</v>
@@ -2728,10 +2714,10 @@
         <v>72</v>
       </c>
       <c r="AV3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AW3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AW3" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="AX3" s="1" t="s">
         <v>72</v>
@@ -2746,19 +2732,19 @@
         <v>72</v>
       </c>
       <c r="BB3" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="BC3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="BC3" s="1" t="s">
-        <v>267</v>
       </c>
       <c r="BD3" s="1" t="s">
         <v>72</v>
       </c>
       <c r="BE3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="BF3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="BF3" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="BG3" s="1" t="s">
         <v>72</v>
@@ -2791,49 +2777,49 @@
         <v>72</v>
       </c>
       <c r="BQ3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="BR3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="BS3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="BT3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="BU3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="BV3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="BW3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="BX3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="BY3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="BZ3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="CA3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="CB3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="BR3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="BS3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="BT3" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="BU3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="BV3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="BW3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="BX3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="BY3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="BZ3" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="CA3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="CB3" s="1" t="s">
-        <v>50</v>
       </c>
       <c r="CC3" s="1" t="s">
         <v>72</v>
       </c>
       <c r="CD3" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="CE3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="CE3" s="1" t="s">
-        <v>268</v>
       </c>
       <c r="CF3" s="1" t="s">
         <v>72</v>
@@ -2857,10 +2843,10 @@
         <v>72</v>
       </c>
       <c r="CM3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="CN3" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="CN3" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="CO3" s="1" t="s">
         <v>72</v>
@@ -2871,11 +2857,8 @@
       <c r="CQ3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="CR3" s="1" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="4" spans="1:96">
+    <row r="4" spans="1:95">
       <c r="A4" s="1" t="s">
         <v>73</v>
       </c>
@@ -2889,49 +2872,49 @@
         <v>76</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>77</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>200</v>
       </c>
       <c r="I4" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="M4" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>281</v>
       </c>
       <c r="T4" s="1" t="s">
         <v>78</v>
@@ -2940,212 +2923,209 @@
         <v>79</v>
       </c>
       <c r="V4" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="X4" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>284</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>208</v>
       </c>
       <c r="Z4" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="AA4" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="AA4" s="1" t="s">
-        <v>207</v>
-      </c>
       <c r="AB4" s="1" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AD4" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>217</v>
+        <v>80</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AG4" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AH4" s="1" t="s">
-        <v>82</v>
+        <v>283</v>
       </c>
       <c r="AI4" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="AJ4" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AK4" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="AJ4" s="1" t="s">
+      <c r="AL4" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="AK4" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="AL4" s="1" t="s">
+      <c r="AM4" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="AM4" s="1" t="s">
+      <c r="AN4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="AO4" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="AN4" s="1" t="s">
+      <c r="AP4" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="AO4" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AP4" s="1" t="s">
+      <c r="AQ4" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="AQ4" s="1" t="s">
+      <c r="AR4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="AS4" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="AR4" s="1" t="s">
+      <c r="AT4" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="AS4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="AT4" s="1" t="s">
+      <c r="AU4" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="AU4" s="1" t="s">
+      <c r="AV4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="AW4" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="AV4" s="1" t="s">
+      <c r="AX4" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="AW4" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="AX4" s="1" t="s">
+      <c r="AY4" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="AY4" s="1" t="s">
+      <c r="AZ4" s="1"/>
+      <c r="BA4" s="1"/>
+      <c r="BB4" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="AZ4" s="1" t="s">
+      <c r="BC4" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="BA4" s="1"/>
-      <c r="BB4" s="1"/>
-      <c r="BC4" s="1" t="s">
+      <c r="BD4" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="BD4" s="1" t="s">
+      <c r="BE4" s="1" t="s">
         <v>300</v>
       </c>
-      <c r="BE4" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="BF4" s="1" t="s">
-        <v>302</v>
-      </c>
+      <c r="BF4" s="1"/>
       <c r="BG4" s="1"/>
       <c r="BH4" s="1"/>
       <c r="BI4" s="1"/>
       <c r="BJ4" s="1"/>
       <c r="BK4" s="1"/>
-      <c r="BL4" s="1"/>
+      <c r="BL4" s="1" t="s">
+        <v>301</v>
+      </c>
       <c r="BM4" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="BN4" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="BN4" s="1" t="s">
+      <c r="BO4" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="BO4" s="1" t="s">
+      <c r="BP4" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="BP4" s="1" t="s">
+      <c r="BQ4" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="BQ4" s="1" t="s">
+      <c r="BR4" s="1" t="s">
         <v>307</v>
       </c>
-      <c r="BR4" s="1" t="s">
+      <c r="BS4" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="BS4" s="1" t="s">
+      <c r="BT4" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="BT4" s="1" t="s">
+      <c r="BU4" s="1" t="s">
         <v>310</v>
       </c>
-      <c r="BU4" s="1" t="s">
+      <c r="BV4" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="BV4" s="1" t="s">
+      <c r="BW4" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="BW4" s="1" t="s">
+      <c r="BX4" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="BX4" s="1" t="s">
+      <c r="BY4" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="BY4" s="1" t="s">
+      <c r="BZ4" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="BZ4" s="1" t="s">
+      <c r="CA4" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="CA4" s="1" t="s">
+      <c r="CB4" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="CB4" s="1" t="s">
+      <c r="CC4" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="CC4" s="1" t="s">
+      <c r="CD4" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="CD4" s="1" t="s">
+      <c r="CE4" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="CE4" s="1" t="s">
+      <c r="CF4" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="CF4" s="1" t="s">
+      <c r="CG4" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="CG4" s="1" t="s">
+      <c r="CH4" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="CH4" s="1" t="s">
+      <c r="CI4" s="1"/>
+      <c r="CJ4" s="1"/>
+      <c r="CK4" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="CI4" s="1" t="s">
+      <c r="CL4" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="CJ4" s="1"/>
-      <c r="CK4" s="1"/>
-      <c r="CL4" s="1" t="s">
+      <c r="CM4" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="CM4" s="1" t="s">
+      <c r="CN4" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="CN4" s="1" t="s">
+      <c r="CO4" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="CO4" s="1" t="s">
-        <v>329</v>
-      </c>
       <c r="CP4" s="1" t="s">
-        <v>330</v>
+        <v>87</v>
       </c>
       <c r="CQ4" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="CR4" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:96">
+    <row r="5" spans="1:95">
       <c r="A5" s="1" t="s">
         <v>89</v>
       </c>
@@ -3192,7 +3172,7 @@
         <v>72</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>72</v>
@@ -3201,7 +3181,7 @@
         <v>72</v>
       </c>
       <c r="S5" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>72</v>
@@ -3225,10 +3205,10 @@
         <v>72</v>
       </c>
       <c r="AA5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AB5" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="AC5" s="1" t="s">
         <v>72</v>
@@ -3243,16 +3223,16 @@
         <v>72</v>
       </c>
       <c r="AG5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI5" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="AJ5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AH5" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI5" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ5" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="AK5" s="1" t="s">
         <v>72</v>
@@ -3261,10 +3241,10 @@
         <v>72</v>
       </c>
       <c r="AM5" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="AN5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AN5" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="AO5" s="1" t="s">
         <v>72</v>
@@ -3273,10 +3253,10 @@
         <v>72</v>
       </c>
       <c r="AQ5" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="AR5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AR5" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="AS5" s="1" t="s">
         <v>72</v>
@@ -3285,10 +3265,10 @@
         <v>72</v>
       </c>
       <c r="AU5" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="AV5" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="AV5" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="AW5" s="1" t="s">
         <v>72</v>
@@ -3297,133 +3277,133 @@
         <v>72</v>
       </c>
       <c r="AY5" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="AZ5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BA5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="AZ5" s="1" t="s">
+      <c r="BB5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BC5" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="BD5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BE5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BF5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BG5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BH5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BI5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BJ5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BK5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BL5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BM5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BN5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BO5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BP5" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="BQ5" s="1" t="s">
         <v>333</v>
       </c>
-      <c r="BA5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BB5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BC5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BD5" s="1" t="s">
+      <c r="BR5" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="BS5" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="BT5" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="BE5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BF5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BG5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BH5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BI5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BJ5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BK5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BL5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BM5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BN5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BO5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BP5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BQ5" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="BR5" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="BS5" s="1" t="s">
-        <v>335</v>
-      </c>
-      <c r="BT5" s="1" t="s">
-        <v>335</v>
-      </c>
       <c r="BU5" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="BV5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="BW5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="BX5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="BY5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="BZ5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="CA5" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="CB5" s="1" t="s">
         <v>335</v>
       </c>
       <c r="CC5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CD5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CE5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CF5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CG5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CH5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CI5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CJ5" s="1" t="s">
-        <v>337</v>
+        <v>201</v>
       </c>
       <c r="CK5" s="1" t="s">
-        <v>201</v>
+        <v>335</v>
       </c>
       <c r="CL5" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="CM5" s="1" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="CN5" s="1" t="s">
         <v>335</v>
       </c>
       <c r="CO5" s="1" t="s">
-        <v>337</v>
+        <v>72</v>
       </c>
       <c r="CP5" s="1" t="s">
         <v>72</v>
@@ -3431,106 +3411,103 @@
       <c r="CQ5" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="CR5" s="1" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="6" spans="1:96">
+    <row r="6" spans="1:95">
       <c r="A6" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="S6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="W6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="X6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z6" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="S6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AA6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AB6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="AC6" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AD6" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AG6" s="1" t="s">
         <v>201</v>
@@ -3542,10 +3519,10 @@
         <v>201</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AL6" s="1" t="s">
         <v>201</v>
@@ -3554,10 +3531,10 @@
         <v>201</v>
       </c>
       <c r="AN6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AP6" s="1" t="s">
         <v>201</v>
@@ -3566,10 +3543,10 @@
         <v>201</v>
       </c>
       <c r="AR6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="AS6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AT6" s="1" t="s">
         <v>201</v>
@@ -3578,10 +3555,10 @@
         <v>201</v>
       </c>
       <c r="AV6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="AW6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="AX6" s="1" t="s">
         <v>201</v>
@@ -3611,22 +3588,22 @@
         <v>201</v>
       </c>
       <c r="BG6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="BH6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="BI6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="BJ6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="BK6" s="1" t="s">
-        <v>201</v>
+        <v>338</v>
       </c>
       <c r="BL6" s="1" t="s">
-        <v>340</v>
+        <v>201</v>
       </c>
       <c r="BM6" s="1" t="s">
         <v>201</v>
@@ -3713,19 +3690,16 @@
         <v>201</v>
       </c>
       <c r="CO6" s="1" t="s">
-        <v>201</v>
+        <v>337</v>
       </c>
       <c r="CP6" s="1" t="s">
-        <v>339</v>
+        <v>201</v>
       </c>
       <c r="CQ6" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR6" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="7" spans="1:96">
+    <row r="7" spans="1:95">
       <c r="A7" s="1" t="s">
         <v>92</v>
       </c>
@@ -3799,7 +3773,7 @@
         <v>201</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>201</v>
@@ -3808,7 +3782,7 @@
         <v>201</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>201</v>
+        <v>94</v>
       </c>
       <c r="AC7" s="1" t="s">
         <v>94</v>
@@ -3817,61 +3791,61 @@
         <v>94</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AF7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AG7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ7" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AL7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN7" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AP7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR7" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU7" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="AT7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU7" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV7" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW7" s="1" t="s">
-        <v>93</v>
+        <v>201</v>
       </c>
       <c r="AX7" s="1" t="s">
         <v>201</v>
@@ -4003,19 +3977,16 @@
         <v>201</v>
       </c>
       <c r="CO7" s="1" t="s">
-        <v>201</v>
+        <v>340</v>
       </c>
       <c r="CP7" s="1" t="s">
-        <v>342</v>
+        <v>201</v>
       </c>
       <c r="CQ7" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR7" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="8" spans="1:96">
+    <row r="8" spans="1:95">
       <c r="A8" s="1" t="s">
         <v>95</v>
       </c>
@@ -4089,7 +4060,7 @@
         <v>201</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="Z8" s="1" t="s">
         <v>201</v>
@@ -4098,7 +4069,7 @@
         <v>201</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="AC8" s="1" t="s">
         <v>97</v>
@@ -4107,61 +4078,61 @@
         <v>97</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AF8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AG8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ8" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AL8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN8" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AP8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR8" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="AT8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU8" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV8" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW8" s="1" t="s">
-        <v>96</v>
+        <v>201</v>
       </c>
       <c r="AX8" s="1" t="s">
         <v>201</v>
@@ -4293,19 +4264,16 @@
         <v>201</v>
       </c>
       <c r="CO8" s="1" t="s">
-        <v>201</v>
+        <v>342</v>
       </c>
       <c r="CP8" s="1" t="s">
-        <v>344</v>
+        <v>201</v>
       </c>
       <c r="CQ8" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR8" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="9" spans="1:96">
+    <row r="9" spans="1:95">
       <c r="A9" s="1" t="s">
         <v>98</v>
       </c>
@@ -4397,61 +4365,61 @@
         <v>201</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="AF9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AG9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ9" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AL9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN9" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AP9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR9" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV9" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="AT9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU9" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV9" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW9" s="1" t="s">
-        <v>99</v>
+        <v>201</v>
       </c>
       <c r="AX9" s="1" t="s">
         <v>201</v>
@@ -4591,11 +4559,8 @@
       <c r="CQ9" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR9" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="10" spans="1:96">
+    <row r="10" spans="1:95">
       <c r="A10" s="1" t="s">
         <v>100</v>
       </c>
@@ -4687,61 +4652,61 @@
         <v>201</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>201</v>
+        <v>94</v>
       </c>
       <c r="AF10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AG10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ10" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AL10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN10" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AP10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR10" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU10" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AT10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU10" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV10" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW10" s="1" t="s">
-        <v>94</v>
+        <v>201</v>
       </c>
       <c r="AX10" s="1" t="s">
         <v>201</v>
@@ -4881,11 +4846,8 @@
       <c r="CQ10" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR10" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="11" spans="1:96">
+    <row r="11" spans="1:95">
       <c r="A11" s="1" t="s">
         <v>101</v>
       </c>
@@ -4977,61 +4939,61 @@
         <v>201</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>201</v>
+        <v>102</v>
       </c>
       <c r="AF11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AG11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ11" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AL11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN11" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AP11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR11" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU11" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AT11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU11" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV11" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW11" s="1" t="s">
-        <v>102</v>
+        <v>201</v>
       </c>
       <c r="AX11" s="1" t="s">
         <v>201</v>
@@ -5171,11 +5133,8 @@
       <c r="CQ11" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR11" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="12" spans="1:96">
+    <row r="12" spans="1:95">
       <c r="A12" s="1" t="s">
         <v>103</v>
       </c>
@@ -5267,61 +5226,61 @@
         <v>201</v>
       </c>
       <c r="AE12" s="1" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="AF12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AG12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ12" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AL12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN12" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AP12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR12" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU12" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV12" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="AT12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU12" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV12" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW12" s="1" t="s">
-        <v>97</v>
+        <v>201</v>
       </c>
       <c r="AX12" s="1" t="s">
         <v>201</v>
@@ -5461,11 +5420,8 @@
       <c r="CQ12" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR12" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="13" spans="1:96">
+    <row r="13" spans="1:95">
       <c r="A13" s="1" t="s">
         <v>104</v>
       </c>
@@ -5557,61 +5513,61 @@
         <v>201</v>
       </c>
       <c r="AE13" s="1" t="s">
-        <v>201</v>
+        <v>105</v>
       </c>
       <c r="AF13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AG13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ13" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AL13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN13" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AP13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR13" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV13" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="AT13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU13" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV13" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW13" s="1" t="s">
-        <v>105</v>
+        <v>201</v>
       </c>
       <c r="AX13" s="1" t="s">
         <v>201</v>
@@ -5751,11 +5707,8 @@
       <c r="CQ13" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR13" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="14" spans="1:96">
+    <row r="14" spans="1:95">
       <c r="A14" s="1" t="s">
         <v>106</v>
       </c>
@@ -5847,61 +5800,61 @@
         <v>201</v>
       </c>
       <c r="AE14" s="1" t="s">
-        <v>201</v>
+        <v>107</v>
       </c>
       <c r="AF14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AG14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AH14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AI14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AJ14" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AG14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AH14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AI14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AJ14" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AK14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AL14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AM14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AN14" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AL14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AM14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN14" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AO14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AP14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AQ14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR14" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AP14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AQ14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AR14" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AS14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AT14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AU14" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="AV14" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AT14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AU14" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="AV14" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="AW14" s="1" t="s">
-        <v>107</v>
+        <v>201</v>
       </c>
       <c r="AX14" s="1" t="s">
         <v>201</v>
@@ -6041,11 +5994,8 @@
       <c r="CQ14" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR14" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="15" spans="1:96">
+    <row r="15" spans="1:95">
       <c r="A15" s="1" t="s">
         <v>108</v>
       </c>
@@ -6152,10 +6102,10 @@
         <v>201</v>
       </c>
       <c r="AJ15" s="1" t="s">
-        <v>201</v>
+        <v>343</v>
       </c>
       <c r="AK15" s="1" t="s">
-        <v>345</v>
+        <v>201</v>
       </c>
       <c r="AL15" s="1" t="s">
         <v>201</v>
@@ -6164,10 +6114,10 @@
         <v>201</v>
       </c>
       <c r="AN15" s="1" t="s">
-        <v>201</v>
+        <v>343</v>
       </c>
       <c r="AO15" s="1" t="s">
-        <v>345</v>
+        <v>201</v>
       </c>
       <c r="AP15" s="1" t="s">
         <v>201</v>
@@ -6176,10 +6126,10 @@
         <v>201</v>
       </c>
       <c r="AR15" s="1" t="s">
-        <v>201</v>
+        <v>343</v>
       </c>
       <c r="AS15" s="1" t="s">
-        <v>345</v>
+        <v>201</v>
       </c>
       <c r="AT15" s="1" t="s">
         <v>201</v>
@@ -6188,10 +6138,10 @@
         <v>201</v>
       </c>
       <c r="AV15" s="1" t="s">
-        <v>201</v>
+        <v>343</v>
       </c>
       <c r="AW15" s="1" t="s">
-        <v>345</v>
+        <v>201</v>
       </c>
       <c r="AX15" s="1" t="s">
         <v>201</v>
@@ -6331,11 +6281,8 @@
       <c r="CQ15" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR15" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="16" spans="1:96">
+    <row r="16" spans="1:95">
       <c r="A16" s="1" t="s">
         <v>109</v>
       </c>
@@ -6621,11 +6568,8 @@
       <c r="CQ16" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR16" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="17" spans="1:96">
+    <row r="17" spans="1:95">
       <c r="A17" s="1" t="s">
         <v>110</v>
       </c>
@@ -6911,11 +6855,8 @@
       <c r="CQ17" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR17" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="18" spans="1:96">
+    <row r="18" spans="1:95">
       <c r="A18" s="1" t="s">
         <v>111</v>
       </c>
@@ -7201,11 +7142,8 @@
       <c r="CQ18" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR18" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="19" spans="1:96">
+    <row r="19" spans="1:95">
       <c r="A19" s="1" t="s">
         <v>112</v>
       </c>
@@ -7491,11 +7429,8 @@
       <c r="CQ19" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR19" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="20" spans="1:96">
+    <row r="20" spans="1:95">
       <c r="A20" s="1" t="s">
         <v>113</v>
       </c>
@@ -7781,11 +7716,8 @@
       <c r="CQ20" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR20" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="21" spans="1:96">
+    <row r="21" spans="1:95">
       <c r="A21" s="1" t="s">
         <v>114</v>
       </c>
@@ -8071,11 +8003,8 @@
       <c r="CQ21" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR21" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="22" spans="1:96">
+    <row r="22" spans="1:95">
       <c r="A22" s="1" t="s">
         <v>115</v>
       </c>
@@ -8361,11 +8290,8 @@
       <c r="CQ22" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR22" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="23" spans="1:96">
+    <row r="23" spans="1:95">
       <c r="A23" s="1" t="s">
         <v>116</v>
       </c>
@@ -8651,11 +8577,8 @@
       <c r="CQ23" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR23" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="24" spans="1:96">
+    <row r="24" spans="1:95">
       <c r="A24" s="1" t="s">
         <v>117</v>
       </c>
@@ -8941,11 +8864,8 @@
       <c r="CQ24" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR24" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="25" spans="1:96">
+    <row r="25" spans="1:95">
       <c r="A25" s="1" t="s">
         <v>118</v>
       </c>
@@ -9231,11 +9151,8 @@
       <c r="CQ25" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR25" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="26" spans="1:96">
+    <row r="26" spans="1:95">
       <c r="A26" s="1" t="s">
         <v>119</v>
       </c>
@@ -9521,11 +9438,8 @@
       <c r="CQ26" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR26" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="27" spans="1:96">
+    <row r="27" spans="1:95">
       <c r="A27" s="1" t="s">
         <v>120</v>
       </c>
@@ -9811,11 +9725,8 @@
       <c r="CQ27" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR27" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="28" spans="1:96">
+    <row r="28" spans="1:95">
       <c r="A28" s="1" t="s">
         <v>121</v>
       </c>
@@ -10101,11 +10012,8 @@
       <c r="CQ28" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR28" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="29" spans="1:96">
+    <row r="29" spans="1:95">
       <c r="A29" s="1" t="s">
         <v>122</v>
       </c>
@@ -10391,11 +10299,8 @@
       <c r="CQ29" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR29" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="30" spans="1:96">
+    <row r="30" spans="1:95">
       <c r="A30" s="1" t="s">
         <v>123</v>
       </c>
@@ -10681,11 +10586,8 @@
       <c r="CQ30" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR30" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="31" spans="1:96">
+    <row r="31" spans="1:95">
       <c r="A31" s="1" t="s">
         <v>124</v>
       </c>
@@ -10971,11 +10873,8 @@
       <c r="CQ31" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR31" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="32" spans="1:96">
+    <row r="32" spans="1:95">
       <c r="A32" s="1" t="s">
         <v>125</v>
       </c>
@@ -11261,11 +11160,8 @@
       <c r="CQ32" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR32" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="33" spans="1:96">
+    <row r="33" spans="1:95">
       <c r="A33" s="1" t="s">
         <v>126</v>
       </c>
@@ -11551,11 +11447,8 @@
       <c r="CQ33" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR33" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="34" spans="1:96">
+    <row r="34" spans="1:95">
       <c r="A34" s="1" t="s">
         <v>127</v>
       </c>
@@ -11841,11 +11734,8 @@
       <c r="CQ34" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR34" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="35" spans="1:96">
+    <row r="35" spans="1:95">
       <c r="A35" s="1" t="s">
         <v>128</v>
       </c>
@@ -12131,11 +12021,8 @@
       <c r="CQ35" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR35" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="36" spans="1:96">
+    <row r="36" spans="1:95">
       <c r="A36" s="1" t="s">
         <v>129</v>
       </c>
@@ -12421,11 +12308,8 @@
       <c r="CQ36" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR36" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="37" spans="1:96">
+    <row r="37" spans="1:95">
       <c r="A37" s="1" t="s">
         <v>130</v>
       </c>
@@ -12711,11 +12595,8 @@
       <c r="CQ37" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR37" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="38" spans="1:96">
+    <row r="38" spans="1:95">
       <c r="A38" s="1" t="s">
         <v>131</v>
       </c>
@@ -13001,11 +12882,8 @@
       <c r="CQ38" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR38" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="39" spans="1:96">
+    <row r="39" spans="1:95">
       <c r="A39" s="1" t="s">
         <v>132</v>
       </c>
@@ -13291,11 +13169,8 @@
       <c r="CQ39" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR39" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="40" spans="1:96">
+    <row r="40" spans="1:95">
       <c r="A40" s="1" t="s">
         <v>133</v>
       </c>
@@ -13581,11 +13456,8 @@
       <c r="CQ40" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR40" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="41" spans="1:96">
+    <row r="41" spans="1:95">
       <c r="A41" s="1" t="s">
         <v>134</v>
       </c>
@@ -13871,11 +13743,8 @@
       <c r="CQ41" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR41" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="42" spans="1:96">
+    <row r="42" spans="1:95">
       <c r="A42" s="1" t="s">
         <v>135</v>
       </c>
@@ -14161,11 +14030,8 @@
       <c r="CQ42" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR42" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="43" spans="1:96">
+    <row r="43" spans="1:95">
       <c r="A43" s="1" t="s">
         <v>136</v>
       </c>
@@ -14451,11 +14317,8 @@
       <c r="CQ43" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR43" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="44" spans="1:96">
+    <row r="44" spans="1:95">
       <c r="A44" s="1" t="s">
         <v>137</v>
       </c>
@@ -14741,11 +14604,8 @@
       <c r="CQ44" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR44" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="45" spans="1:96">
+    <row r="45" spans="1:95">
       <c r="A45" s="1" t="s">
         <v>138</v>
       </c>
@@ -15031,11 +14891,8 @@
       <c r="CQ45" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR45" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="46" spans="1:96">
+    <row r="46" spans="1:95">
       <c r="A46" s="1" t="s">
         <v>139</v>
       </c>
@@ -15321,11 +15178,8 @@
       <c r="CQ46" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR46" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="47" spans="1:96">
+    <row r="47" spans="1:95">
       <c r="A47" s="1" t="s">
         <v>140</v>
       </c>
@@ -15611,11 +15465,8 @@
       <c r="CQ47" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR47" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="48" spans="1:96">
+    <row r="48" spans="1:95">
       <c r="A48" s="1" t="s">
         <v>141</v>
       </c>
@@ -15901,11 +15752,8 @@
       <c r="CQ48" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR48" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="49" spans="1:96">
+    <row r="49" spans="1:95">
       <c r="A49" s="1" t="s">
         <v>142</v>
       </c>
@@ -16191,11 +16039,8 @@
       <c r="CQ49" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR49" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="50" spans="1:96">
+    <row r="50" spans="1:95">
       <c r="A50" s="1" t="s">
         <v>143</v>
       </c>
@@ -16481,11 +16326,8 @@
       <c r="CQ50" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR50" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="51" spans="1:96">
+    <row r="51" spans="1:95">
       <c r="A51" s="1" t="s">
         <v>144</v>
       </c>
@@ -16771,11 +16613,8 @@
       <c r="CQ51" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR51" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="52" spans="1:96">
+    <row r="52" spans="1:95">
       <c r="A52" s="1" t="s">
         <v>145</v>
       </c>
@@ -17061,11 +16900,8 @@
       <c r="CQ52" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR52" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="53" spans="1:96">
+    <row r="53" spans="1:95">
       <c r="A53" s="1" t="s">
         <v>146</v>
       </c>
@@ -17351,11 +17187,8 @@
       <c r="CQ53" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR53" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="54" spans="1:96">
+    <row r="54" spans="1:95">
       <c r="A54" s="1" t="s">
         <v>147</v>
       </c>
@@ -17641,11 +17474,8 @@
       <c r="CQ54" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR54" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="55" spans="1:96">
+    <row r="55" spans="1:95">
       <c r="A55" s="1" t="s">
         <v>148</v>
       </c>
@@ -17931,11 +17761,8 @@
       <c r="CQ55" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR55" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="56" spans="1:96">
+    <row r="56" spans="1:95">
       <c r="A56" s="1" t="s">
         <v>149</v>
       </c>
@@ -18221,11 +18048,8 @@
       <c r="CQ56" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR56" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="57" spans="1:96">
+    <row r="57" spans="1:95">
       <c r="A57" s="1" t="s">
         <v>150</v>
       </c>
@@ -18511,11 +18335,8 @@
       <c r="CQ57" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR57" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="58" spans="1:96">
+    <row r="58" spans="1:95">
       <c r="A58" s="1" t="s">
         <v>151</v>
       </c>
@@ -18801,11 +18622,8 @@
       <c r="CQ58" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR58" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="59" spans="1:96">
+    <row r="59" spans="1:95">
       <c r="A59" s="1" t="s">
         <v>152</v>
       </c>
@@ -19091,11 +18909,8 @@
       <c r="CQ59" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR59" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="60" spans="1:96">
+    <row r="60" spans="1:95">
       <c r="A60" s="1" t="s">
         <v>153</v>
       </c>
@@ -19381,11 +19196,8 @@
       <c r="CQ60" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR60" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="61" spans="1:96">
+    <row r="61" spans="1:95">
       <c r="A61" s="1" t="s">
         <v>154</v>
       </c>
@@ -19671,11 +19483,8 @@
       <c r="CQ61" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR61" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="62" spans="1:96">
+    <row r="62" spans="1:95">
       <c r="A62" s="1" t="s">
         <v>155</v>
       </c>
@@ -19961,11 +19770,8 @@
       <c r="CQ62" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR62" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="63" spans="1:96">
+    <row r="63" spans="1:95">
       <c r="A63" s="1" t="s">
         <v>156</v>
       </c>
@@ -20251,11 +20057,8 @@
       <c r="CQ63" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR63" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="64" spans="1:96">
+    <row r="64" spans="1:95">
       <c r="A64" s="1" t="s">
         <v>157</v>
       </c>
@@ -20541,11 +20344,8 @@
       <c r="CQ64" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR64" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="65" spans="1:96">
+    <row r="65" spans="1:95">
       <c r="A65" s="1" t="s">
         <v>158</v>
       </c>
@@ -20831,11 +20631,8 @@
       <c r="CQ65" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR65" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="66" spans="1:96">
+    <row r="66" spans="1:95">
       <c r="A66" s="1" t="s">
         <v>159</v>
       </c>
@@ -21121,11 +20918,8 @@
       <c r="CQ66" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR66" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="67" spans="1:96">
+    <row r="67" spans="1:95">
       <c r="A67" s="1" t="s">
         <v>160</v>
       </c>
@@ -21411,11 +21205,8 @@
       <c r="CQ67" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR67" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="68" spans="1:96">
+    <row r="68" spans="1:95">
       <c r="A68" s="1" t="s">
         <v>161</v>
       </c>
@@ -21701,11 +21492,8 @@
       <c r="CQ68" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR68" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="69" spans="1:96">
+    <row r="69" spans="1:95">
       <c r="A69" s="1" t="s">
         <v>162</v>
       </c>
@@ -21991,11 +21779,8 @@
       <c r="CQ69" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR69" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="70" spans="1:96">
+    <row r="70" spans="1:95">
       <c r="A70" s="1" t="s">
         <v>163</v>
       </c>
@@ -22281,11 +22066,8 @@
       <c r="CQ70" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR70" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="71" spans="1:96">
+    <row r="71" spans="1:95">
       <c r="A71" s="1" t="s">
         <v>164</v>
       </c>
@@ -22571,11 +22353,8 @@
       <c r="CQ71" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR71" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="72" spans="1:96">
+    <row r="72" spans="1:95">
       <c r="A72" s="1" t="s">
         <v>165</v>
       </c>
@@ -22861,11 +22640,8 @@
       <c r="CQ72" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR72" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="73" spans="1:96">
+    <row r="73" spans="1:95">
       <c r="A73" s="1" t="s">
         <v>166</v>
       </c>
@@ -23151,11 +22927,8 @@
       <c r="CQ73" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR73" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="74" spans="1:96">
+    <row r="74" spans="1:95">
       <c r="A74" s="1" t="s">
         <v>167</v>
       </c>
@@ -23441,11 +23214,8 @@
       <c r="CQ74" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR74" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="75" spans="1:96">
+    <row r="75" spans="1:95">
       <c r="A75" s="1" t="s">
         <v>168</v>
       </c>
@@ -23731,11 +23501,8 @@
       <c r="CQ75" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR75" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="76" spans="1:96">
+    <row r="76" spans="1:95">
       <c r="A76" s="1" t="s">
         <v>169</v>
       </c>
@@ -24021,11 +23788,8 @@
       <c r="CQ76" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR76" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="77" spans="1:96">
+    <row r="77" spans="1:95">
       <c r="A77" s="1" t="s">
         <v>170</v>
       </c>
@@ -24311,11 +24075,8 @@
       <c r="CQ77" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR77" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="78" spans="1:96">
+    <row r="78" spans="1:95">
       <c r="A78" s="1" t="s">
         <v>171</v>
       </c>
@@ -24601,11 +24362,8 @@
       <c r="CQ78" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR78" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="79" spans="1:96">
+    <row r="79" spans="1:95">
       <c r="A79" s="1" t="s">
         <v>172</v>
       </c>
@@ -24891,11 +24649,8 @@
       <c r="CQ79" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR79" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="80" spans="1:96">
+    <row r="80" spans="1:95">
       <c r="A80" s="1" t="s">
         <v>173</v>
       </c>
@@ -25181,11 +24936,8 @@
       <c r="CQ80" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR80" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="81" spans="1:96">
+    <row r="81" spans="1:95">
       <c r="A81" s="1" t="s">
         <v>174</v>
       </c>
@@ -25471,11 +25223,8 @@
       <c r="CQ81" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR81" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="82" spans="1:96">
+    <row r="82" spans="1:95">
       <c r="A82" s="1" t="s">
         <v>175</v>
       </c>
@@ -25761,11 +25510,8 @@
       <c r="CQ82" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR82" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="83" spans="1:96">
+    <row r="83" spans="1:95">
       <c r="A83" s="1" t="s">
         <v>176</v>
       </c>
@@ -26051,11 +25797,8 @@
       <c r="CQ83" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR83" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="84" spans="1:96">
+    <row r="84" spans="1:95">
       <c r="A84" s="1" t="s">
         <v>177</v>
       </c>
@@ -26341,11 +26084,8 @@
       <c r="CQ84" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR84" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="85" spans="1:96">
+    <row r="85" spans="1:95">
       <c r="A85" s="1" t="s">
         <v>178</v>
       </c>
@@ -26631,11 +26371,8 @@
       <c r="CQ85" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR85" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="86" spans="1:96">
+    <row r="86" spans="1:95">
       <c r="A86" s="1" t="s">
         <v>179</v>
       </c>
@@ -26921,11 +26658,8 @@
       <c r="CQ86" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR86" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="87" spans="1:96">
+    <row r="87" spans="1:95">
       <c r="A87" s="1" t="s">
         <v>180</v>
       </c>
@@ -27211,11 +26945,8 @@
       <c r="CQ87" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR87" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="88" spans="1:96">
+    <row r="88" spans="1:95">
       <c r="A88" s="1" t="s">
         <v>181</v>
       </c>
@@ -27501,11 +27232,8 @@
       <c r="CQ88" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR88" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="89" spans="1:96">
+    <row r="89" spans="1:95">
       <c r="A89" s="1" t="s">
         <v>182</v>
       </c>
@@ -27791,11 +27519,8 @@
       <c r="CQ89" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR89" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="90" spans="1:96">
+    <row r="90" spans="1:95">
       <c r="A90" s="1" t="s">
         <v>183</v>
       </c>
@@ -28081,11 +27806,8 @@
       <c r="CQ90" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR90" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="91" spans="1:96">
+    <row r="91" spans="1:95">
       <c r="A91" s="1" t="s">
         <v>184</v>
       </c>
@@ -28371,11 +28093,8 @@
       <c r="CQ91" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR91" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="92" spans="1:96">
+    <row r="92" spans="1:95">
       <c r="A92" s="1" t="s">
         <v>185</v>
       </c>
@@ -28661,11 +28380,8 @@
       <c r="CQ92" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR92" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="93" spans="1:96">
+    <row r="93" spans="1:95">
       <c r="A93" s="1" t="s">
         <v>186</v>
       </c>
@@ -28951,11 +28667,8 @@
       <c r="CQ93" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR93" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="94" spans="1:96">
+    <row r="94" spans="1:95">
       <c r="A94" s="1" t="s">
         <v>187</v>
       </c>
@@ -29241,11 +28954,8 @@
       <c r="CQ94" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR94" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="95" spans="1:96">
+    <row r="95" spans="1:95">
       <c r="A95" s="1" t="s">
         <v>188</v>
       </c>
@@ -29531,11 +29241,8 @@
       <c r="CQ95" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR95" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="96" spans="1:96">
+    <row r="96" spans="1:95">
       <c r="A96" s="1" t="s">
         <v>189</v>
       </c>
@@ -29821,11 +29528,8 @@
       <c r="CQ96" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR96" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="97" spans="1:96">
+    <row r="97" spans="1:95">
       <c r="A97" s="1" t="s">
         <v>190</v>
       </c>
@@ -30111,11 +29815,8 @@
       <c r="CQ97" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR97" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="98" spans="1:96">
+    <row r="98" spans="1:95">
       <c r="A98" s="1" t="s">
         <v>191</v>
       </c>
@@ -30401,11 +30102,8 @@
       <c r="CQ98" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR98" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="99" spans="1:96">
+    <row r="99" spans="1:95">
       <c r="A99" s="1" t="s">
         <v>192</v>
       </c>
@@ -30691,11 +30389,8 @@
       <c r="CQ99" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR99" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="100" spans="1:96">
+    <row r="100" spans="1:95">
       <c r="A100" s="1" t="s">
         <v>193</v>
       </c>
@@ -30981,11 +30676,8 @@
       <c r="CQ100" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR100" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="101" spans="1:96">
+    <row r="101" spans="1:95">
       <c r="A101" s="1" t="s">
         <v>194</v>
       </c>
@@ -31271,11 +30963,8 @@
       <c r="CQ101" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR101" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="102" spans="1:96">
+    <row r="102" spans="1:95">
       <c r="A102" s="1" t="s">
         <v>195</v>
       </c>
@@ -31561,11 +31250,8 @@
       <c r="CQ102" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR102" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="103" spans="1:96">
+    <row r="103" spans="1:95">
       <c r="A103" s="1" t="s">
         <v>196</v>
       </c>
@@ -31851,11 +31537,8 @@
       <c r="CQ103" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR103" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="104" spans="1:96">
+    <row r="104" spans="1:95">
       <c r="A104" s="1" t="s">
         <v>197</v>
       </c>
@@ -32141,11 +31824,8 @@
       <c r="CQ104" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR104" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="105" spans="1:96">
+    <row r="105" spans="1:95">
       <c r="A105" s="1" t="s">
         <v>198</v>
       </c>
@@ -32431,11 +32111,8 @@
       <c r="CQ105" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="CR105" s="1" t="s">
-        <v>201</v>
-      </c>
     </row>
-    <row r="106" spans="1:96">
+    <row r="106" spans="1:95">
       <c r="A106" s="1" t="s">
         <v>199</v>
       </c>
@@ -32719,16 +32396,13 @@
         <v>201</v>
       </c>
       <c r="CQ106" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="CR106" s="1" t="s">
         <v>201</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:CR6" xr:uid="{1E35D5F4-5515-4605-A6EE-F624486B4945}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:CQ6" xr:uid="{1E35D5F4-5515-4605-A6EE-F624486B4945}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
         <mc:Choice Requires="x12ac">
           <x12ac:list>"yes,no,-"</x12ac:list>

</xml_diff>

<commit_message>
Rename substrate_1_type and substrate_1_mg to substrate_type and substrate_mg
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_results/lanupro_vocabulary_incubations.xlsx
+++ b/data/raw_results/lanupro_vocabulary_incubations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my_github_projects\lanupro_vocabulary_2025\data\raw_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7F43F5-6E6B-4196-8C12-BEC699D74FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB1B0264-E051-40A9-8BD5-A402DB7F0944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7197A02B-EEB4-4DD3-A670-5499E50D1EFE}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10060" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10060" uniqueCount="346">
   <si>
     <t>lanupro_ontology</t>
   </si>
@@ -1098,6 +1098,12 @@
   </si>
   <si>
     <t>sc</t>
+  </si>
+  <si>
+    <t>substrate_type</t>
+  </si>
+  <si>
+    <t>substrate_mg</t>
   </si>
 </sst>
 </file>
@@ -1557,8 +1563,8 @@
     <tableColumn id="91" xr3:uid="{4C65E12D-86B9-473B-A866-FE3129457F9C}" uniqueName="91" name="cow_ilvo_id" queryTableFieldId="101"/>
     <tableColumn id="92" xr3:uid="{B28188A6-01B4-4D1F-A64D-7AE40B7F5845}" uniqueName="92" name="diet_cows" queryTableFieldId="102"/>
     <tableColumn id="79" xr3:uid="{5DDB981D-3A78-45F3-8EC2-94928028E554}" uniqueName="79" name="inocula_type" queryTableFieldId="81"/>
-    <tableColumn id="80" xr3:uid="{A01C1450-87EF-47A3-9093-B7C7EACE4000}" uniqueName="80" name="substrate_1_type" queryTableFieldId="82"/>
-    <tableColumn id="73" xr3:uid="{F985F988-5F8F-4A6F-8482-53D9E7052230}" uniqueName="73" name="substrate_1_mg" queryTableFieldId="89"/>
+    <tableColumn id="80" xr3:uid="{A01C1450-87EF-47A3-9093-B7C7EACE4000}" uniqueName="80" name="substrate_type" queryTableFieldId="82"/>
+    <tableColumn id="73" xr3:uid="{F985F988-5F8F-4A6F-8482-53D9E7052230}" uniqueName="73" name="substrate_mg" queryTableFieldId="89"/>
     <tableColumn id="15" xr3:uid="{6C1AE535-1B92-4BEE-A9B7-C36F9C205E82}" uniqueName="15" name="trt_label_1" queryTableFieldId="15" dataDxfId="63"/>
     <tableColumn id="77" xr3:uid="{D3AEC664-491F-49A5-A9F2-35E0EDEC2C61}" uniqueName="77" name="trt_label_2" queryTableFieldId="79" dataDxfId="62"/>
     <tableColumn id="78" xr3:uid="{DACCF43A-F357-4C51-9B95-DCD03E783460}" uniqueName="78" name="trt_label_3" queryTableFieldId="80" dataDxfId="61"/>
@@ -2074,10 +2080,10 @@
         <v>202</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>210</v>
+        <v>344</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>211</v>
+        <v>345</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>212</v>
@@ -2648,10 +2654,10 @@
         <v>72</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>72</v>
+        <v>210</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>72</v>
+        <v>211</v>
       </c>
       <c r="AB3" s="1" t="s">
         <v>72</v>

</xml_diff>